<commit_message>
Add PDF guide, update lab files and user DB
Add a PDF version of the DevSecOps lab guide and refresh related lab assets. Added Guias_de_Laboratorio/Guia_Lab_U3_S9_DevSecOps_Fork.pdf, updated the .docx, and removed the .gitkeep placeholder. Also updated Administracion/Lista_Asistencia_ASS_CRN236396.xlsx and refreshed the devsecops lab users DB (devsecops-lab/app/users.db). These changes publish the guide in PDF form and update attendance and user data for the lab.
</commit_message>
<xml_diff>
--- a/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
+++ b/Administracion/Lista_Asistencia_ASS_CRN236396.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5ddf5fb2bc65e958/Documentos/GitHub/lc_arquitectura_de_sistemas_de_seguridad/Administracion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="14_{545CCF96-C524-4C47-965E-B405D4770607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F14BD334-306E-456D-A0E5-B0C5F4E3E279}"/>
+  <xr:revisionPtr revIDLastSave="129" documentId="14_{545CCF96-C524-4C47-965E-B405D4770607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56960807-9F25-4073-AF78-1FEDF67E0AE4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1274,7 +1274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1349,40 +1349,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1418,6 +1399,24 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1743,94 +1742,94 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28"/>
-      <c r="T1" s="28"/>
-      <c r="U1" s="28"/>
-      <c r="V1" s="28"/>
-      <c r="W1" s="28"/>
-      <c r="X1" s="28"/>
-      <c r="Y1" s="28"/>
-      <c r="Z1" s="28"/>
-      <c r="AA1" s="28"/>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="28"/>
-      <c r="AD1" s="28"/>
-      <c r="AE1" s="28"/>
-      <c r="AF1" s="28"/>
-      <c r="AG1" s="28"/>
-      <c r="AH1" s="28"/>
-      <c r="AI1" s="28"/>
-      <c r="AJ1" s="28"/>
-      <c r="AK1" s="28"/>
-      <c r="AL1" s="28"/>
-      <c r="AM1" s="28"/>
-      <c r="AN1" s="28"/>
-      <c r="AO1" s="28"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="49"/>
+      <c r="K1" s="49"/>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="49"/>
+      <c r="Q1" s="49"/>
+      <c r="R1" s="49"/>
+      <c r="S1" s="49"/>
+      <c r="T1" s="49"/>
+      <c r="U1" s="49"/>
+      <c r="V1" s="49"/>
+      <c r="W1" s="49"/>
+      <c r="X1" s="49"/>
+      <c r="Y1" s="49"/>
+      <c r="Z1" s="49"/>
+      <c r="AA1" s="49"/>
+      <c r="AB1" s="49"/>
+      <c r="AC1" s="49"/>
+      <c r="AD1" s="49"/>
+      <c r="AE1" s="49"/>
+      <c r="AF1" s="49"/>
+      <c r="AG1" s="49"/>
+      <c r="AH1" s="49"/>
+      <c r="AI1" s="49"/>
+      <c r="AJ1" s="49"/>
+      <c r="AK1" s="49"/>
+      <c r="AL1" s="49"/>
+      <c r="AM1" s="49"/>
+      <c r="AN1" s="49"/>
+      <c r="AO1" s="49"/>
     </row>
     <row r="2" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-      <c r="K2" s="29"/>
-      <c r="L2" s="29"/>
-      <c r="M2" s="29"/>
-      <c r="N2" s="29"/>
-      <c r="O2" s="29"/>
-      <c r="P2" s="29"/>
-      <c r="Q2" s="29"/>
-      <c r="R2" s="29"/>
-      <c r="S2" s="29"/>
-      <c r="T2" s="29"/>
-      <c r="U2" s="29"/>
-      <c r="V2" s="29"/>
-      <c r="W2" s="29"/>
-      <c r="X2" s="29"/>
-      <c r="Y2" s="29"/>
-      <c r="Z2" s="29"/>
-      <c r="AA2" s="29"/>
-      <c r="AB2" s="29"/>
-      <c r="AC2" s="29"/>
-      <c r="AD2" s="29"/>
-      <c r="AE2" s="29"/>
-      <c r="AF2" s="29"/>
-      <c r="AG2" s="29"/>
-      <c r="AH2" s="29"/>
-      <c r="AI2" s="29"/>
-      <c r="AJ2" s="29"/>
-      <c r="AK2" s="29"/>
-      <c r="AL2" s="29"/>
-      <c r="AM2" s="29"/>
-      <c r="AN2" s="29"/>
-      <c r="AO2" s="29"/>
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
+      <c r="M2" s="50"/>
+      <c r="N2" s="50"/>
+      <c r="O2" s="50"/>
+      <c r="P2" s="50"/>
+      <c r="Q2" s="50"/>
+      <c r="R2" s="50"/>
+      <c r="S2" s="50"/>
+      <c r="T2" s="50"/>
+      <c r="U2" s="50"/>
+      <c r="V2" s="50"/>
+      <c r="W2" s="50"/>
+      <c r="X2" s="50"/>
+      <c r="Y2" s="50"/>
+      <c r="Z2" s="50"/>
+      <c r="AA2" s="50"/>
+      <c r="AB2" s="50"/>
+      <c r="AC2" s="50"/>
+      <c r="AD2" s="50"/>
+      <c r="AE2" s="50"/>
+      <c r="AF2" s="50"/>
+      <c r="AG2" s="50"/>
+      <c r="AH2" s="50"/>
+      <c r="AI2" s="50"/>
+      <c r="AJ2" s="50"/>
+      <c r="AK2" s="50"/>
+      <c r="AL2" s="50"/>
+      <c r="AM2" s="50"/>
+      <c r="AN2" s="50"/>
+      <c r="AO2" s="50"/>
     </row>
     <row r="3" spans="1:41" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -1851,70 +1850,70 @@
       <c r="F3" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="G3" s="30" t="s">
+      <c r="G3" s="45" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="30"/>
-      <c r="I3" s="31" t="s">
+      <c r="H3" s="45"/>
+      <c r="I3" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="31"/>
-      <c r="K3" s="30" t="s">
+      <c r="J3" s="46"/>
+      <c r="K3" s="45" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="30"/>
-      <c r="M3" s="31" t="s">
+      <c r="L3" s="45"/>
+      <c r="M3" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="N3" s="31"/>
-      <c r="O3" s="30" t="s">
+      <c r="N3" s="46"/>
+      <c r="O3" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="31" t="s">
+      <c r="P3" s="45"/>
+      <c r="Q3" s="46" t="s">
         <v>11</v>
       </c>
-      <c r="R3" s="31"/>
-      <c r="S3" s="30" t="s">
+      <c r="R3" s="46"/>
+      <c r="S3" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="T3" s="30"/>
-      <c r="U3" s="31" t="s">
+      <c r="T3" s="45"/>
+      <c r="U3" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="V3" s="31"/>
-      <c r="W3" s="30" t="s">
+      <c r="V3" s="46"/>
+      <c r="W3" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="31" t="s">
+      <c r="X3" s="45"/>
+      <c r="Y3" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="Z3" s="31"/>
-      <c r="AA3" s="30" t="s">
+      <c r="Z3" s="46"/>
+      <c r="AA3" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="AB3" s="30"/>
-      <c r="AC3" s="31" t="s">
+      <c r="AB3" s="45"/>
+      <c r="AC3" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="AD3" s="31"/>
-      <c r="AE3" s="30" t="s">
+      <c r="AD3" s="46"/>
+      <c r="AE3" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="AF3" s="30"/>
-      <c r="AG3" s="31" t="s">
+      <c r="AF3" s="45"/>
+      <c r="AG3" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="AH3" s="31"/>
-      <c r="AI3" s="30" t="s">
+      <c r="AH3" s="46"/>
+      <c r="AI3" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="AJ3" s="30"/>
-      <c r="AK3" s="31" t="s">
+      <c r="AJ3" s="45"/>
+      <c r="AK3" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="AL3" s="31"/>
+      <c r="AL3" s="46"/>
       <c r="AM3" s="4" t="s">
         <v>22</v>
       </c>
@@ -2607,7 +2606,7 @@
         <v>73</v>
       </c>
       <c r="E10" s="11">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F10" s="11">
         <f>IFERROR(ROUND(_xlfn.XLOOKUP(B10&amp;" "&amp;C10,'Examen 1'!B$2:B$27,'Examen 1'!E$2:E$27,0)/100*5,1),0)</f>
@@ -3844,115 +3843,115 @@
         <v>0.6875</v>
       </c>
     </row>
-    <row r="21" spans="1:41" s="39" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="34">
+    <row r="21" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="28">
         <v>16</v>
       </c>
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="29" t="s">
         <v>105</v>
       </c>
-      <c r="D21" s="36" t="s">
+      <c r="D21" s="30" t="s">
         <v>106</v>
       </c>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36">
+      <c r="E21" s="30"/>
+      <c r="F21" s="30">
         <f>IFERROR(ROUND(_xlfn.XLOOKUP(B21&amp;" "&amp;C21,'Examen 1'!B$2:B$27,'Examen 1'!E$2:E$27,0)/100*5,1),0)</f>
         <v>5</v>
       </c>
-      <c r="G21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="H21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="I21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="J21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="K21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="L21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="M21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="N21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="O21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="P21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="Q21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="R21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="S21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="T21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="U21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="V21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="W21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="X21" s="37" t="s">
+      <c r="G21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="H21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="J21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="K21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="L21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="M21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="N21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="O21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="P21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="R21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="S21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="T21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="U21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="V21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="W21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="X21" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="Y21" s="37" t="s">
+      <c r="Y21" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="Z21" s="37" t="s">
+      <c r="Z21" s="31" t="s">
         <v>146</v>
       </c>
-      <c r="AA21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="AB21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="AC21" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="AD21" s="37" t="s">
+      <c r="AA21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="AB21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="AC21" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="AD21" s="31" t="s">
         <v>145</v>
       </c>
       <c r="AE21" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="AF21" s="37"/>
-      <c r="AG21" s="40"/>
-      <c r="AH21" s="37"/>
-      <c r="AI21" s="37"/>
-      <c r="AJ21" s="37"/>
-      <c r="AK21" s="37"/>
-      <c r="AL21" s="37"/>
-      <c r="AM21" s="34">
+      <c r="AF21" s="31"/>
+      <c r="AG21" s="33"/>
+      <c r="AH21" s="31"/>
+      <c r="AI21" s="31"/>
+      <c r="AJ21" s="31"/>
+      <c r="AK21" s="31"/>
+      <c r="AL21" s="31"/>
+      <c r="AM21" s="28">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="AN21" s="34">
+      <c r="AN21" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="AO21" s="38">
+      <c r="AO21" s="32">
         <f t="shared" si="2"/>
         <v>0.6875</v>
       </c>
@@ -4536,7 +4535,7 @@
         <v>124</v>
       </c>
       <c r="E27" s="18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27" s="11">
         <f>IFERROR(ROUND(_xlfn.XLOOKUP(B27&amp;" "&amp;C27,'Examen 1'!B$2:B$27,'Examen 1'!E$2:E$27,0)/100*5,1),0)</f>
@@ -4764,7 +4763,7 @@
         <v>130</v>
       </c>
       <c r="E29" s="18">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="F29" s="11">
         <f>IFERROR(ROUND(_xlfn.XLOOKUP(B29&amp;" "&amp;C29,'Examen 1'!B$2:B$27,'Examen 1'!E$2:E$27,0)/100*5,1),0)</f>
@@ -5211,12 +5210,12 @@
       </c>
     </row>
     <row r="33" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32" t="s">
+      <c r="A33" s="47" t="s">
         <v>140</v>
       </c>
-      <c r="B33" s="32"/>
-      <c r="C33" s="32"/>
-      <c r="D33" s="32"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="47"/>
+      <c r="D33" s="47"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="20">
@@ -5352,49 +5351,49 @@
       <c r="AO33" s="5"/>
     </row>
     <row r="34" spans="1:41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="33" t="s">
+      <c r="A34" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="33"/>
-      <c r="C34" s="33"/>
-      <c r="D34" s="33"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="33"/>
-      <c r="G34" s="33"/>
-      <c r="H34" s="33"/>
-      <c r="I34" s="33"/>
-      <c r="J34" s="33"/>
-      <c r="K34" s="33"/>
-      <c r="L34" s="33"/>
-      <c r="M34" s="33"/>
-      <c r="N34" s="33"/>
-      <c r="O34" s="33"/>
-      <c r="P34" s="33"/>
-      <c r="Q34" s="33"/>
-      <c r="R34" s="33"/>
-      <c r="S34" s="33"/>
-      <c r="T34" s="33"/>
-      <c r="U34" s="33"/>
-      <c r="V34" s="33"/>
-      <c r="W34" s="33"/>
-      <c r="X34" s="33"/>
-      <c r="Y34" s="33"/>
-      <c r="Z34" s="33"/>
-      <c r="AA34" s="33"/>
-      <c r="AB34" s="33"/>
-      <c r="AC34" s="33"/>
-      <c r="AD34" s="33"/>
-      <c r="AE34" s="33"/>
-      <c r="AF34" s="33"/>
-      <c r="AG34" s="33"/>
-      <c r="AH34" s="33"/>
-      <c r="AI34" s="33"/>
-      <c r="AJ34" s="33"/>
-      <c r="AK34" s="33"/>
-      <c r="AL34" s="33"/>
-      <c r="AM34" s="33"/>
-      <c r="AN34" s="33"/>
-      <c r="AO34" s="33"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="48"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="48"/>
+      <c r="L34" s="48"/>
+      <c r="M34" s="48"/>
+      <c r="N34" s="48"/>
+      <c r="O34" s="48"/>
+      <c r="P34" s="48"/>
+      <c r="Q34" s="48"/>
+      <c r="R34" s="48"/>
+      <c r="S34" s="48"/>
+      <c r="T34" s="48"/>
+      <c r="U34" s="48"/>
+      <c r="V34" s="48"/>
+      <c r="W34" s="48"/>
+      <c r="X34" s="48"/>
+      <c r="Y34" s="48"/>
+      <c r="Z34" s="48"/>
+      <c r="AA34" s="48"/>
+      <c r="AB34" s="48"/>
+      <c r="AC34" s="48"/>
+      <c r="AD34" s="48"/>
+      <c r="AE34" s="48"/>
+      <c r="AF34" s="48"/>
+      <c r="AG34" s="48"/>
+      <c r="AH34" s="48"/>
+      <c r="AI34" s="48"/>
+      <c r="AJ34" s="48"/>
+      <c r="AK34" s="48"/>
+      <c r="AL34" s="48"/>
+      <c r="AM34" s="48"/>
+      <c r="AN34" s="48"/>
+      <c r="AO34" s="48"/>
     </row>
     <row r="35" spans="1:41" x14ac:dyDescent="0.25">
       <c r="AG35" s="26" t="s">
@@ -5403,6 +5402,10 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="AA3:AB3"/>
+    <mergeCell ref="AC3:AD3"/>
+    <mergeCell ref="AE3:AF3"/>
+    <mergeCell ref="AG3:AH3"/>
     <mergeCell ref="AI3:AJ3"/>
     <mergeCell ref="AK3:AL3"/>
     <mergeCell ref="A33:D33"/>
@@ -5419,10 +5422,6 @@
     <mergeCell ref="U3:V3"/>
     <mergeCell ref="W3:X3"/>
     <mergeCell ref="Y3:Z3"/>
-    <mergeCell ref="AA3:AB3"/>
-    <mergeCell ref="AC3:AD3"/>
-    <mergeCell ref="AE3:AF3"/>
-    <mergeCell ref="AG3:AH3"/>
   </mergeCells>
   <conditionalFormatting sqref="AO6:AO32">
     <cfRule type="expression" dxfId="1" priority="2">
@@ -5452,16 +5451,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="49" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
@@ -6321,2269 +6320,2269 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="B1" s="41" t="s">
+      <c r="B1" s="34" t="s">
         <v>276</v>
       </c>
-      <c r="C1" s="41" t="s">
+      <c r="C1" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="D1" s="41" t="s">
+      <c r="D1" s="34" t="s">
         <v>273</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="F1" s="41" t="s">
+      <c r="F1" s="34" t="s">
         <v>151</v>
       </c>
-      <c r="G1" s="41" t="s">
+      <c r="G1" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="H1" s="41" t="s">
+      <c r="H1" s="34" t="s">
         <v>153</v>
       </c>
-      <c r="I1" s="41" t="s">
+      <c r="I1" s="34" t="s">
         <v>154</v>
       </c>
-      <c r="J1" s="41" t="s">
+      <c r="J1" s="34" t="s">
         <v>155</v>
       </c>
-      <c r="K1" s="41" t="s">
+      <c r="K1" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="L1" s="41" t="s">
+      <c r="L1" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="M1" s="41" t="s">
+      <c r="M1" s="34" t="s">
         <v>158</v>
       </c>
-      <c r="N1" s="41" t="s">
+      <c r="N1" s="34" t="s">
         <v>159</v>
       </c>
-      <c r="O1" s="41" t="s">
+      <c r="O1" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="P1" s="41" t="s">
+      <c r="P1" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="Q1" s="41" t="s">
+      <c r="Q1" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="R1" s="41" t="s">
+      <c r="R1" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="S1" s="41" t="s">
+      <c r="S1" s="34" t="s">
         <v>164</v>
       </c>
-      <c r="T1" s="41" t="s">
+      <c r="T1" s="34" t="s">
         <v>165</v>
       </c>
-      <c r="U1" s="41" t="s">
+      <c r="U1" s="34" t="s">
         <v>166</v>
       </c>
-      <c r="V1" s="41" t="s">
+      <c r="V1" s="34" t="s">
         <v>167</v>
       </c>
-      <c r="W1" s="41" t="s">
+      <c r="W1" s="34" t="s">
         <v>168</v>
       </c>
-      <c r="X1" s="41" t="s">
+      <c r="X1" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="Y1" s="41" t="s">
+      <c r="Y1" s="34" t="s">
         <v>170</v>
       </c>
-      <c r="Z1" s="41" t="s">
+      <c r="Z1" s="34" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" s="43">
+      <c r="A2" s="36">
         <v>46106.414525462962</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="36" t="s">
         <v>277</v>
       </c>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="D2" s="45" t="s">
+      <c r="D2" s="38" t="s">
         <v>181</v>
       </c>
-      <c r="E2" s="46">
+      <c r="E2" s="39">
         <f>MIN(100,VALUE(TRIM(LEFT(D2,FIND("/",D2)-1))))</f>
         <v>94</v>
       </c>
-      <c r="F2" s="44" t="s">
+      <c r="F2" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G2" s="44" t="s">
+      <c r="G2" s="37" t="s">
         <v>183</v>
       </c>
-      <c r="H2" s="44" t="s">
+      <c r="H2" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I2" s="44" t="s">
+      <c r="I2" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J2" s="44" t="s">
+      <c r="J2" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K2" s="44" t="s">
+      <c r="K2" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L2" s="44" t="s">
+      <c r="L2" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M2" s="44" t="s">
+      <c r="M2" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N2" s="44" t="s">
+      <c r="N2" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O2" s="44" t="s">
+      <c r="O2" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="W2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y2" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z2" s="44" t="s">
+      <c r="P2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q2" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T2" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="V2" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="W2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X2" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y2" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z2" s="37" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" s="47">
+      <c r="A3" s="40">
         <v>46106.414560185185</v>
       </c>
-      <c r="B3" s="47" t="s">
+      <c r="B3" s="40" t="s">
         <v>278</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="41" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="49" t="s">
+      <c r="D3" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E3" s="46">
+      <c r="E3" s="39">
         <f t="shared" ref="E3:E28" si="0">MIN(100,VALUE(TRIM(LEFT(D3,FIND("/",D3)-1))))</f>
         <v>100</v>
       </c>
-      <c r="F3" s="48" t="s">
+      <c r="F3" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G3" s="48" t="s">
+      <c r="G3" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H3" s="48" t="s">
+      <c r="H3" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I3" s="48" t="s">
+      <c r="I3" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J3" s="48" t="s">
+      <c r="J3" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K3" s="48" t="s">
+      <c r="K3" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L3" s="48" t="s">
+      <c r="L3" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M3" s="48" t="s">
+      <c r="M3" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N3" s="48" t="s">
+      <c r="N3" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O3" s="48" t="s">
+      <c r="O3" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q3" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T3" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U3" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X3" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y3" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z3" s="48" t="s">
+      <c r="P3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q3" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T3" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U3" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X3" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y3" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z3" s="41" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" s="43">
+      <c r="A4" s="36">
         <v>46106.41511574074</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="36" t="s">
         <v>279</v>
       </c>
-      <c r="C4" s="44" t="s">
+      <c r="C4" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="E4" s="46">
+      <c r="E4" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F4" s="44" t="s">
+      <c r="F4" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H4" s="44" t="s">
+      <c r="H4" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I4" s="44" t="s">
+      <c r="I4" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J4" s="44" t="s">
+      <c r="J4" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K4" s="44" t="s">
+      <c r="K4" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L4" s="44" t="s">
+      <c r="L4" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M4" s="44" t="s">
+      <c r="M4" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N4" s="44" t="s">
+      <c r="N4" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O4" s="44" t="s">
+      <c r="O4" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q4" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T4" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U4" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X4" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y4" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z4" s="44" t="s">
+      <c r="P4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q4" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T4" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U4" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X4" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y4" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z4" s="37" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" s="47">
+      <c r="A5" s="40">
         <v>46106.416435185187</v>
       </c>
-      <c r="B5" s="47" t="s">
+      <c r="B5" s="40" t="s">
         <v>280</v>
       </c>
-      <c r="C5" s="48" t="s">
+      <c r="C5" s="41" t="s">
         <v>198</v>
       </c>
-      <c r="D5" s="49" t="s">
+      <c r="D5" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="E5" s="46">
+      <c r="E5" s="39">
         <f t="shared" si="0"/>
         <v>88</v>
       </c>
-      <c r="F5" s="48" t="s">
+      <c r="F5" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H5" s="48" t="s">
+      <c r="H5" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I5" s="48" t="s">
+      <c r="I5" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J5" s="48" t="s">
+      <c r="J5" s="41" t="s">
         <v>200</v>
       </c>
-      <c r="K5" s="48" t="s">
+      <c r="K5" s="41" t="s">
         <v>201</v>
       </c>
-      <c r="L5" s="48" t="s">
+      <c r="L5" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M5" s="48" t="s">
+      <c r="M5" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N5" s="48" t="s">
+      <c r="N5" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O5" s="48" t="s">
+      <c r="O5" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q5" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T5" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="V5" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="W5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X5" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y5" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z5" s="48" t="s">
+      <c r="P5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q5" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T5" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="V5" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="W5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X5" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y5" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z5" s="41" t="s">
         <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" s="43">
+      <c r="A6" s="36">
         <v>46106.416608796295</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="B6" s="36" t="s">
         <v>281</v>
       </c>
-      <c r="C6" s="44" t="s">
+      <c r="C6" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="38" t="s">
         <v>204</v>
       </c>
-      <c r="E6" s="46">
+      <c r="E6" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F6" s="44" t="s">
+      <c r="F6" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G6" s="44" t="s">
+      <c r="G6" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H6" s="44" t="s">
+      <c r="H6" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I6" s="44" t="s">
+      <c r="I6" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J6" s="44" t="s">
+      <c r="J6" s="37" t="s">
         <v>200</v>
       </c>
-      <c r="K6" s="44" t="s">
+      <c r="K6" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L6" s="44" t="s">
+      <c r="L6" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M6" s="44" t="s">
+      <c r="M6" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N6" s="44" t="s">
+      <c r="N6" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O6" s="44" t="s">
+      <c r="O6" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q6" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T6" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U6" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X6" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y6" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z6" s="44" t="s">
+      <c r="P6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q6" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T6" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U6" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X6" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y6" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z6" s="37" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" s="47">
+      <c r="A7" s="40">
         <v>46106.417118055557</v>
       </c>
-      <c r="B7" s="47" t="s">
+      <c r="B7" s="40" t="s">
         <v>282</v>
       </c>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="41" t="s">
         <v>206</v>
       </c>
-      <c r="D7" s="49" t="s">
+      <c r="D7" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E7" s="46">
+      <c r="E7" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F7" s="48" t="s">
+      <c r="F7" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G7" s="48" t="s">
+      <c r="G7" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H7" s="48" t="s">
+      <c r="H7" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I7" s="48" t="s">
+      <c r="I7" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J7" s="48" t="s">
+      <c r="J7" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K7" s="48" t="s">
+      <c r="K7" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M7" s="48" t="s">
+      <c r="M7" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N7" s="48" t="s">
+      <c r="N7" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O7" s="48" t="s">
+      <c r="O7" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q7" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T7" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U7" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X7" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y7" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z7" s="48" t="s">
+      <c r="P7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q7" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T7" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U7" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X7" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y7" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z7" s="41" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" s="43">
+      <c r="A8" s="36">
         <v>46106.417129629626</v>
       </c>
-      <c r="B8" s="43" t="s">
+      <c r="B8" s="36" t="s">
         <v>283</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="37" t="s">
         <v>208</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="E8" s="46">
+      <c r="E8" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F8" s="44" t="s">
+      <c r="F8" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I8" s="44" t="s">
+      <c r="I8" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J8" s="44" t="s">
+      <c r="J8" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K8" s="44" t="s">
+      <c r="K8" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L8" s="44" t="s">
+      <c r="L8" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M8" s="44" t="s">
+      <c r="M8" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N8" s="44" t="s">
+      <c r="N8" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O8" s="44" t="s">
+      <c r="O8" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q8" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T8" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U8" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X8" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y8" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z8" s="44" t="s">
+      <c r="P8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q8" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T8" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U8" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X8" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y8" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z8" s="37" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" s="47">
+      <c r="A9" s="40">
         <v>46106.417349537034</v>
       </c>
-      <c r="B9" s="47" t="s">
+      <c r="B9" s="40" t="s">
         <v>284</v>
       </c>
-      <c r="C9" s="48" t="s">
+      <c r="C9" s="41" t="s">
         <v>210</v>
       </c>
-      <c r="D9" s="49" t="s">
+      <c r="D9" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E9" s="46">
+      <c r="E9" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F9" s="48" t="s">
+      <c r="F9" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I9" s="48" t="s">
+      <c r="I9" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J9" s="48" t="s">
+      <c r="J9" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K9" s="48" t="s">
+      <c r="K9" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L9" s="48" t="s">
+      <c r="L9" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M9" s="48" t="s">
+      <c r="M9" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N9" s="48" t="s">
+      <c r="N9" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O9" s="48" t="s">
+      <c r="O9" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q9" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T9" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U9" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X9" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y9" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z9" s="48" t="s">
+      <c r="P9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q9" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T9" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U9" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X9" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y9" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z9" s="41" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" s="43">
+      <c r="A10" s="36">
         <v>46106.418194444443</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="C10" s="44" t="s">
+      <c r="C10" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="38" t="s">
         <v>213</v>
       </c>
-      <c r="E10" s="46">
+      <c r="E10" s="39">
         <f t="shared" si="0"/>
         <v>90</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="H10" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I10" s="44" t="s">
+      <c r="I10" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J10" s="44" t="s">
+      <c r="J10" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K10" s="44" t="s">
+      <c r="K10" s="37" t="s">
         <v>215</v>
       </c>
-      <c r="L10" s="44" t="s">
+      <c r="L10" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M10" s="44" t="s">
+      <c r="M10" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N10" s="44" t="s">
+      <c r="N10" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O10" s="44" t="s">
+      <c r="O10" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q10" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="U10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X10" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y10" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z10" s="44" t="s">
+      <c r="P10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q10" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="U10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="V10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X10" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y10" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z10" s="37" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" s="47">
+      <c r="A11" s="40">
         <v>46106.418958333335</v>
       </c>
-      <c r="B11" s="47" t="s">
+      <c r="B11" s="40" t="s">
         <v>286</v>
       </c>
-      <c r="C11" s="48" t="s">
+      <c r="C11" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="D11" s="49" t="s">
+      <c r="D11" s="42" t="s">
         <v>218</v>
       </c>
-      <c r="E11" s="46">
+      <c r="E11" s="39">
         <f t="shared" si="0"/>
         <v>98</v>
       </c>
-      <c r="F11" s="48" t="s">
+      <c r="F11" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G11" s="48" t="s">
+      <c r="G11" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H11" s="48" t="s">
+      <c r="H11" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I11" s="48" t="s">
+      <c r="I11" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J11" s="48" t="s">
+      <c r="J11" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K11" s="48" t="s">
+      <c r="K11" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L11" s="48" t="s">
+      <c r="L11" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="M11" s="48" t="s">
+      <c r="M11" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N11" s="48" t="s">
+      <c r="N11" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O11" s="48" t="s">
+      <c r="O11" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q11" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T11" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="V11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X11" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y11" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z11" s="48" t="s">
+      <c r="P11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q11" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T11" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="V11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X11" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y11" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z11" s="41" t="s">
         <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" s="43">
+      <c r="A12" s="36">
         <v>46106.418981481482</v>
       </c>
-      <c r="B12" s="43" t="s">
+      <c r="B12" s="36" t="s">
         <v>287</v>
       </c>
-      <c r="C12" s="44" t="s">
+      <c r="C12" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="D12" s="45" t="s">
+      <c r="D12" s="38" t="s">
         <v>222</v>
       </c>
-      <c r="E12" s="46">
+      <c r="E12" s="39">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="F12" s="44" t="s">
+      <c r="F12" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G12" s="44" t="s">
+      <c r="G12" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="H12" s="44" t="s">
+      <c r="H12" s="37" t="s">
         <v>173</v>
       </c>
-      <c r="I12" s="44" t="s">
+      <c r="I12" s="37" t="s">
         <v>224</v>
       </c>
-      <c r="J12" s="44" t="s">
+      <c r="J12" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K12" s="44" t="s">
+      <c r="K12" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L12" s="44" t="s">
+      <c r="L12" s="37" t="s">
         <v>176</v>
       </c>
-      <c r="M12" s="44" t="s">
+      <c r="M12" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N12" s="44" t="s">
+      <c r="N12" s="37" t="s">
         <v>177</v>
       </c>
-      <c r="O12" s="44" t="s">
+      <c r="O12" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P12" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="S12" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="W12" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X12" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y12" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z12" s="44" t="s">
+      <c r="P12" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="S12" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="W12" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X12" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y12" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z12" s="37" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" s="47">
+      <c r="A13" s="40">
         <v>46106.419062499997</v>
       </c>
-      <c r="B13" s="47" t="s">
+      <c r="B13" s="40" t="s">
         <v>288</v>
       </c>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="41" t="s">
         <v>226</v>
       </c>
-      <c r="D13" s="49" t="s">
+      <c r="D13" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="E13" s="46">
+      <c r="E13" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F13" s="48" t="s">
+      <c r="F13" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G13" s="48" t="s">
+      <c r="G13" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H13" s="48" t="s">
+      <c r="H13" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I13" s="48" t="s">
+      <c r="I13" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J13" s="48" t="s">
+      <c r="J13" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K13" s="48" t="s">
+      <c r="K13" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L13" s="48" t="s">
+      <c r="L13" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M13" s="48" t="s">
+      <c r="M13" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N13" s="48" t="s">
+      <c r="N13" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O13" s="48" t="s">
+      <c r="O13" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q13" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="U13" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X13" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y13" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z13" s="48" t="s">
+      <c r="P13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q13" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="U13" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X13" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y13" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z13" s="41" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" s="45" t="s">
+      <c r="A14" s="38" t="s">
         <v>229</v>
       </c>
-      <c r="B14" s="45" t="s">
+      <c r="B14" s="38" t="s">
         <v>289</v>
       </c>
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="37" t="s">
         <v>230</v>
       </c>
-      <c r="D14" s="45" t="s">
+      <c r="D14" s="38" t="s">
         <v>231</v>
       </c>
-      <c r="E14" s="46">
+      <c r="E14" s="39">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="F14" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="G14" s="44" t="s">
+      <c r="G14" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="H14" s="44" t="s">
+      <c r="H14" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I14" s="44" t="s">
+      <c r="I14" s="37" t="s">
         <v>224</v>
       </c>
-      <c r="J14" s="44" t="s">
+      <c r="J14" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K14" s="44" t="s">
+      <c r="K14" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L14" s="44" t="s">
+      <c r="L14" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="M14" s="44" t="s">
+      <c r="M14" s="37" t="s">
         <v>233</v>
       </c>
-      <c r="N14" s="44" t="s">
+      <c r="N14" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O14" s="44" t="s">
+      <c r="O14" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="P14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q14" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S14" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="T14" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V14" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="W14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X14" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y14" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z14" s="44" t="s">
+      <c r="P14" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q14" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R14" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S14" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="T14" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U14" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="V14" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="W14" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X14" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y14" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z14" s="37" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A15" s="47">
+      <c r="A15" s="40">
         <v>46106.419988425929</v>
       </c>
-      <c r="B15" s="47" t="s">
+      <c r="B15" s="40" t="s">
         <v>290</v>
       </c>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="41" t="s">
         <v>236</v>
       </c>
-      <c r="D15" s="49" t="s">
+      <c r="D15" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E15" s="46">
+      <c r="E15" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F15" s="48" t="s">
+      <c r="F15" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G15" s="48" t="s">
+      <c r="G15" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H15" s="48" t="s">
+      <c r="H15" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I15" s="48" t="s">
+      <c r="I15" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J15" s="48" t="s">
+      <c r="J15" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K15" s="48" t="s">
+      <c r="K15" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L15" s="48" t="s">
+      <c r="L15" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M15" s="48" t="s">
+      <c r="M15" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N15" s="48" t="s">
+      <c r="N15" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O15" s="48" t="s">
+      <c r="O15" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q15" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T15" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U15" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X15" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y15" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z15" s="48" t="s">
+      <c r="P15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q15" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T15" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U15" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X15" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y15" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z15" s="41" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A16" s="43">
+      <c r="A16" s="36">
         <v>46106.420046296298</v>
       </c>
-      <c r="B16" s="43" t="s">
+      <c r="B16" s="36" t="s">
         <v>291</v>
       </c>
-      <c r="C16" s="44" t="s">
+      <c r="C16" s="37" t="s">
         <v>238</v>
       </c>
-      <c r="D16" s="45" t="s">
+      <c r="D16" s="38" t="s">
         <v>239</v>
       </c>
-      <c r="E16" s="46">
+      <c r="E16" s="39">
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
-      <c r="F16" s="44" t="s">
+      <c r="F16" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G16" s="44" t="s">
+      <c r="G16" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="H16" s="44" t="s">
+      <c r="H16" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I16" s="44" t="s">
+      <c r="I16" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J16" s="44" t="s">
+      <c r="J16" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K16" s="44" t="s">
+      <c r="K16" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L16" s="44" t="s">
+      <c r="L16" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M16" s="44" t="s">
+      <c r="M16" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N16" s="44" t="s">
+      <c r="N16" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O16" s="44" t="s">
+      <c r="O16" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q16" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="U16" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V16" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="W16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Y16" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z16" s="44" t="s">
+      <c r="P16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q16" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="U16" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V16" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="W16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y16" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z16" s="37" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A17" s="47">
+      <c r="A17" s="40">
         <v>46106.420104166667</v>
       </c>
-      <c r="B17" s="47" t="s">
+      <c r="B17" s="40" t="s">
         <v>292</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="41" t="s">
         <v>241</v>
       </c>
-      <c r="D17" s="49" t="s">
+      <c r="D17" s="42" t="s">
         <v>242</v>
       </c>
-      <c r="E17" s="46">
+      <c r="E17" s="39">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
-      <c r="F17" s="48" t="s">
+      <c r="F17" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G17" s="48" t="s">
+      <c r="G17" s="41" t="s">
         <v>223</v>
       </c>
-      <c r="H17" s="48" t="s">
+      <c r="H17" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I17" s="48" t="s">
+      <c r="I17" s="41" t="s">
         <v>243</v>
       </c>
-      <c r="J17" s="48" t="s">
+      <c r="J17" s="41" t="s">
         <v>214</v>
       </c>
-      <c r="K17" s="48" t="s">
+      <c r="K17" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L17" s="48" t="s">
+      <c r="L17" s="41" t="s">
         <v>219</v>
       </c>
-      <c r="M17" s="48" t="s">
+      <c r="M17" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N17" s="48" t="s">
+      <c r="N17" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O17" s="48" t="s">
+      <c r="O17" s="41" t="s">
         <v>234</v>
       </c>
-      <c r="P17" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="S17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="T17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="W17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="X17" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y17" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z17" s="48" t="s">
+      <c r="P17" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="S17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="T17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="W17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="X17" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y17" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z17" s="41" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A18" s="43">
+      <c r="A18" s="36">
         <v>46106.420347222222</v>
       </c>
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="36" t="s">
         <v>293</v>
       </c>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="37" t="s">
         <v>245</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="E18" s="46">
+      <c r="E18" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F18" s="44" t="s">
+      <c r="F18" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G18" s="44" t="s">
+      <c r="G18" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H18" s="44" t="s">
+      <c r="H18" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J18" s="44" t="s">
+      <c r="J18" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K18" s="44" t="s">
+      <c r="K18" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L18" s="44" t="s">
+      <c r="L18" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M18" s="44" t="s">
+      <c r="M18" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N18" s="44" t="s">
+      <c r="N18" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O18" s="44" t="s">
+      <c r="O18" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q18" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T18" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U18" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X18" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y18" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z18" s="44" t="s">
+      <c r="P18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q18" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T18" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U18" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X18" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y18" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z18" s="37" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A19" s="47">
+      <c r="A19" s="40">
         <v>46106.42046296296</v>
       </c>
-      <c r="B19" s="47" t="s">
+      <c r="B19" s="40" t="s">
         <v>294</v>
       </c>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="41" t="s">
         <v>247</v>
       </c>
-      <c r="D19" s="49" t="s">
+      <c r="D19" s="42" t="s">
         <v>248</v>
       </c>
-      <c r="E19" s="46">
+      <c r="E19" s="39">
         <f t="shared" si="0"/>
         <v>96</v>
       </c>
-      <c r="F19" s="48" t="s">
+      <c r="F19" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G19" s="48" t="s">
+      <c r="G19" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H19" s="48" t="s">
+      <c r="H19" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I19" s="48" t="s">
+      <c r="I19" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J19" s="48" t="s">
+      <c r="J19" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K19" s="48" t="s">
+      <c r="K19" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L19" s="48" t="s">
+      <c r="L19" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M19" s="48" t="s">
+      <c r="M19" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N19" s="48" t="s">
+      <c r="N19" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O19" s="48" t="s">
+      <c r="O19" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P19" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q19" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R19" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="S19" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="T19" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="U19" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V19" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W19" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X19" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y19" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z19" s="48" t="s">
+      <c r="P19" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="S19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="T19" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="U19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V19" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W19" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y19" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z19" s="41" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A20" s="45" t="s">
+      <c r="A20" s="38" t="s">
         <v>250</v>
       </c>
-      <c r="B20" s="45" t="s">
+      <c r="B20" s="38" t="s">
         <v>295</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="C20" s="37" t="s">
         <v>251</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D20" s="38" t="s">
         <v>192</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F20" s="44" t="s">
+      <c r="F20" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G20" s="44" t="s">
+      <c r="G20" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H20" s="44" t="s">
+      <c r="H20" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I20" s="44" t="s">
+      <c r="I20" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J20" s="44" t="s">
+      <c r="J20" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K20" s="44" t="s">
+      <c r="K20" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L20" s="44" t="s">
+      <c r="L20" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M20" s="44" t="s">
+      <c r="M20" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N20" s="44" t="s">
+      <c r="N20" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O20" s="44" t="s">
+      <c r="O20" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q20" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T20" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U20" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X20" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y20" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z20" s="44" t="s">
+      <c r="P20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q20" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T20" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U20" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X20" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y20" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z20" s="37" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="21" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A21" s="47">
+      <c r="A21" s="40">
         <v>46106.421365740738</v>
       </c>
-      <c r="B21" s="47" t="s">
+      <c r="B21" s="40" t="s">
         <v>296</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" s="41" t="s">
         <v>253</v>
       </c>
-      <c r="D21" s="49" t="s">
+      <c r="D21" s="42" t="s">
         <v>254</v>
       </c>
-      <c r="E21" s="46">
+      <c r="E21" s="39">
         <f t="shared" si="0"/>
         <v>77</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G21" s="48" t="s">
+      <c r="G21" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H21" s="48" t="s">
+      <c r="H21" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I21" s="48" t="s">
+      <c r="I21" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J21" s="48" t="s">
+      <c r="J21" s="41" t="s">
         <v>214</v>
       </c>
-      <c r="K21" s="48" t="s">
+      <c r="K21" s="41" t="s">
         <v>172</v>
       </c>
-      <c r="L21" s="48" t="s">
+      <c r="L21" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M21" s="48" t="s">
+      <c r="M21" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N21" s="48" t="s">
+      <c r="N21" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O21" s="48" t="s">
+      <c r="O21" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q21" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R21" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="S21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="U21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="V21" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="W21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Y21" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z21" s="48" t="s">
+      <c r="P21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q21" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R21" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="S21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="U21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="V21" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="W21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y21" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z21" s="41" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="22" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A22" s="43">
+      <c r="A22" s="36">
         <v>46106.422662037039</v>
       </c>
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="36" t="s">
         <v>297</v>
       </c>
-      <c r="C22" s="44" t="s">
+      <c r="C22" s="37" t="s">
         <v>256</v>
       </c>
-      <c r="D22" s="45" t="s">
+      <c r="D22" s="38" t="s">
         <v>257</v>
       </c>
-      <c r="E22" s="46">
+      <c r="E22" s="39">
         <f t="shared" si="0"/>
         <v>66</v>
       </c>
-      <c r="F22" s="44" t="s">
+      <c r="F22" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="G22" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H22" s="44" t="s">
+      <c r="H22" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I22" s="44" t="s">
+      <c r="I22" s="37" t="s">
         <v>243</v>
       </c>
-      <c r="J22" s="44" t="s">
+      <c r="J22" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K22" s="44" t="s">
+      <c r="K22" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="L22" s="44" t="s">
+      <c r="L22" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="M22" s="44" t="s">
+      <c r="M22" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N22" s="44" t="s">
+      <c r="N22" s="37" t="s">
         <v>258</v>
       </c>
-      <c r="O22" s="44" t="s">
+      <c r="O22" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P22" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q22" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R22" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S22" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T22" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U22" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V22" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="W22" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="X22" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y22" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z22" s="44" t="s">
+      <c r="P22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q22" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T22" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="V22" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="W22" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="X22" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y22" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z22" s="37" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="23" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A23" s="47">
+      <c r="A23" s="40">
         <v>46106.42291666667</v>
       </c>
-      <c r="B23" s="47" t="s">
+      <c r="B23" s="40" t="s">
         <v>298</v>
       </c>
-      <c r="C23" s="48" t="s">
+      <c r="C23" s="41" t="s">
         <v>260</v>
       </c>
-      <c r="D23" s="49" t="s">
+      <c r="D23" s="42" t="s">
         <v>192</v>
       </c>
-      <c r="E23" s="46">
+      <c r="E23" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F23" s="48" t="s">
+      <c r="F23" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G23" s="48" t="s">
+      <c r="G23" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H23" s="48" t="s">
+      <c r="H23" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J23" s="48" t="s">
+      <c r="J23" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K23" s="48" t="s">
+      <c r="K23" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L23" s="48" t="s">
+      <c r="L23" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M23" s="48" t="s">
+      <c r="M23" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N23" s="48" t="s">
+      <c r="N23" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O23" s="48" t="s">
+      <c r="O23" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q23" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T23" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U23" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X23" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y23" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z23" s="48" t="s">
+      <c r="P23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q23" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T23" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U23" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X23" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y23" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z23" s="41" t="s">
         <v>261</v>
       </c>
     </row>
     <row r="24" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A24" s="43">
+      <c r="A24" s="36">
         <v>46106.423321759263</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="36" t="s">
         <v>299</v>
       </c>
-      <c r="C24" s="44" t="s">
+      <c r="C24" s="37" t="s">
         <v>262</v>
       </c>
-      <c r="D24" s="45" t="s">
+      <c r="D24" s="38" t="s">
         <v>239</v>
       </c>
-      <c r="E24" s="46">
+      <c r="E24" s="39">
         <f t="shared" si="0"/>
         <v>85</v>
       </c>
-      <c r="F24" s="44" t="s">
+      <c r="F24" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="G24" s="44" t="s">
+      <c r="G24" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H24" s="44" t="s">
+      <c r="H24" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I24" s="44" t="s">
+      <c r="I24" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J24" s="44" t="s">
+      <c r="J24" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K24" s="44" t="s">
+      <c r="K24" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="L24" s="44" t="s">
+      <c r="L24" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M24" s="44" t="s">
+      <c r="M24" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N24" s="44" t="s">
+      <c r="N24" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O24" s="44" t="s">
+      <c r="O24" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q24" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="U24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="V24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X24" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y24" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z24" s="44" t="s">
+      <c r="P24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q24" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="U24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="V24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X24" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y24" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z24" s="37" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="25" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A25" s="47">
+      <c r="A25" s="40">
         <v>46106.443576388891</v>
       </c>
-      <c r="B25" s="47" t="s">
+      <c r="B25" s="40" t="s">
         <v>300</v>
       </c>
-      <c r="C25" s="48" t="s">
+      <c r="C25" s="41" t="s">
         <v>264</v>
       </c>
-      <c r="D25" s="49" t="s">
+      <c r="D25" s="42" t="s">
         <v>265</v>
       </c>
-      <c r="E25" s="46">
+      <c r="E25" s="39">
         <f t="shared" si="0"/>
         <v>99</v>
       </c>
-      <c r="F25" s="48" t="s">
+      <c r="F25" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G25" s="48" t="s">
+      <c r="G25" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H25" s="48" t="s">
+      <c r="H25" s="41" t="s">
         <v>173</v>
       </c>
-      <c r="I25" s="48" t="s">
+      <c r="I25" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J25" s="48" t="s">
+      <c r="J25" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K25" s="48" t="s">
+      <c r="K25" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L25" s="48" t="s">
+      <c r="L25" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M25" s="48" t="s">
+      <c r="M25" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N25" s="48" t="s">
+      <c r="N25" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O25" s="48" t="s">
+      <c r="O25" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P25" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q25" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R25" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S25" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T25" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U25" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V25" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W25" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X25" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y25" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z25" s="48" t="s">
+      <c r="P25" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q25" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R25" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S25" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T25" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U25" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V25" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W25" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X25" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y25" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z25" s="41" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A26" s="43">
+      <c r="A26" s="36">
         <v>46106.445543981485</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="36" t="s">
         <v>301</v>
       </c>
-      <c r="C26" s="44" t="s">
+      <c r="C26" s="37" t="s">
         <v>267</v>
       </c>
-      <c r="D26" s="45" t="s">
+      <c r="D26" s="38" t="s">
         <v>248</v>
       </c>
-      <c r="E26" s="46">
+      <c r="E26" s="39">
         <f t="shared" si="0"/>
         <v>96</v>
       </c>
-      <c r="F26" s="44" t="s">
+      <c r="F26" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G26" s="44" t="s">
+      <c r="G26" s="37" t="s">
         <v>223</v>
       </c>
-      <c r="H26" s="44" t="s">
+      <c r="H26" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I26" s="44" t="s">
+      <c r="I26" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J26" s="44" t="s">
+      <c r="J26" s="37" t="s">
         <v>214</v>
       </c>
-      <c r="K26" s="44" t="s">
+      <c r="K26" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L26" s="44" t="s">
+      <c r="L26" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M26" s="44" t="s">
+      <c r="M26" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N26" s="44" t="s">
+      <c r="N26" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O26" s="44" t="s">
+      <c r="O26" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q26" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T26" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U26" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X26" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y26" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z26" s="44" t="s">
+      <c r="P26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q26" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T26" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U26" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X26" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y26" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z26" s="37" t="s">
         <v>268</v>
       </c>
     </row>
     <row r="27" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A27" s="49" t="s">
+      <c r="A27" s="42" t="s">
         <v>269</v>
       </c>
-      <c r="B27" s="49" t="s">
+      <c r="B27" s="42" t="s">
         <v>302</v>
       </c>
-      <c r="C27" s="48" t="s">
+      <c r="C27" s="41" t="s">
         <v>270</v>
       </c>
-      <c r="D27" s="49" t="s">
+      <c r="D27" s="42" t="s">
         <v>271</v>
       </c>
-      <c r="E27" s="46">
+      <c r="E27" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F27" s="48" t="s">
+      <c r="F27" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="G27" s="48" t="s">
+      <c r="G27" s="41" t="s">
         <v>193</v>
       </c>
-      <c r="H27" s="48" t="s">
+      <c r="H27" s="41" t="s">
         <v>184</v>
       </c>
-      <c r="I27" s="48" t="s">
+      <c r="I27" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="J27" s="48" t="s">
+      <c r="J27" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="K27" s="48" t="s">
+      <c r="K27" s="41" t="s">
         <v>185</v>
       </c>
-      <c r="L27" s="48" t="s">
+      <c r="L27" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="M27" s="48" t="s">
+      <c r="M27" s="41" t="s">
         <v>187</v>
       </c>
-      <c r="N27" s="48" t="s">
+      <c r="N27" s="41" t="s">
         <v>188</v>
       </c>
-      <c r="O27" s="48" t="s">
+      <c r="O27" s="41" t="s">
         <v>189</v>
       </c>
-      <c r="P27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q27" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="R27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="S27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="T27" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="U27" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="V27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="W27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="X27" s="48" t="s">
-        <v>179</v>
-      </c>
-      <c r="Y27" s="48" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z27" s="48" t="s">
+      <c r="P27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q27" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="R27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="S27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="T27" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="U27" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="V27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="W27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="X27" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="Y27" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z27" s="41" t="s">
         <v>272</v>
       </c>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A28" s="43">
+      <c r="A28" s="36">
         <v>46139.668900462966</v>
       </c>
-      <c r="B28" s="50" t="s">
+      <c r="B28" s="43" t="s">
         <v>306</v>
       </c>
-      <c r="C28" s="44" t="s">
+      <c r="C28" s="37" t="s">
         <v>303</v>
       </c>
-      <c r="D28" s="51" t="s">
+      <c r="D28" s="44" t="s">
         <v>304</v>
       </c>
-      <c r="E28" s="46">
+      <c r="E28" s="39">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F28" s="44" t="s">
+      <c r="F28" s="37" t="s">
         <v>182</v>
       </c>
-      <c r="G28" s="44" t="s">
+      <c r="G28" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="H28" s="44" t="s">
+      <c r="H28" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I28" s="44" t="s">
+      <c r="I28" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="J28" s="44" t="s">
+      <c r="J28" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="K28" s="44" t="s">
+      <c r="K28" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="L28" s="44" t="s">
+      <c r="L28" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="M28" s="44" t="s">
+      <c r="M28" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="N28" s="44" t="s">
+      <c r="N28" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="O28" s="44" t="s">
+      <c r="O28" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="P28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Q28" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="R28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="S28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="T28" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="U28" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="V28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="W28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="X28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Y28" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="Z28" s="44" t="s">
+      <c r="P28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q28" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="R28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="S28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="T28" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="U28" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="V28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="W28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="X28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Y28" s="37" t="s">
+        <v>178</v>
+      </c>
+      <c r="Z28" s="37" t="s">
         <v>305</v>
       </c>
     </row>

</xml_diff>